<commit_message>
Reordenar SCORM y sumar entrega final y foro en todos los módulos
</commit_message>
<xml_diff>
--- a/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
+++ b/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
@@ -13,10 +13,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opciones modulares" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Criterios'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Certificación completa'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Base común modular'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opciones modulares'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Criterios'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Certificación completa'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Base común modular'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opciones modulares'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +37,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
@@ -69,7 +68,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -441,14 +442,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Criterio</t>
@@ -478,72 +479,96 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>17 semanas; orden de la planilla original.</t>
+          <t>21 semanas. Anatomía → SCORM → Metáfora → Podcast → Streaming → Simulaciones.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Recorrido por módulos</t>
+          <t>Base común modular</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>4 semanas de base común + un módulo específico.</t>
+          <t>7 semanas: Anatomía, SCORM y Metáfora.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Semanas de trabajo final</t>
+          <t>Entrega final</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Podcast: 1 adicional; Streaming: 1 adicional. Incluidas en los totales.</t>
+          <t>1 semana adicional en cada módulo, incluida en todos los totales.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Recesos</t>
+          <t>Foros</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>No contemplados; semanas consecutivas de martes a lunes.</t>
+          <t>Todos los módulos incluyen un foro de intercambio.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Disponibilidad</t>
+          <t>Proyecto de certificación</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Calendario estimado; no representa el estado de producción de abril.</t>
+          <t>Diseño de un objeto de aprendizaje propio.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Articulación del proyecto</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente de definir su relación con trabajos de módulo; sin semana integradora adicional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Recesos</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>No contemplados; semanas consecutivas de martes a lunes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Acreditación modular</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Denominación institucional pendiente.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -554,19 +579,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Módulo</t>
@@ -574,17 +602,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Duración (semanas)</t>
+          <t>Cursada (semanas)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Semana inicial</t>
+          <t>Entrega (semanas)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Semana final</t>
+          <t>Total del módulo</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -594,12 +622,27 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Fin de cursada</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Criterio / producción</t>
+          <t>Inicio de entrega</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Fin de entrega</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Foro</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Total de trayectoria</t>
         </is>
       </c>
     </row>
@@ -616,7 +659,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>46126</v>
@@ -624,149 +667,191 @@
       <c r="F2" s="3" t="n">
         <v>46132</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Reconocer los componentes de un objeto de aprendizaje.</t>
-        </is>
-      </c>
+      <c r="G2" s="3" t="n">
+        <v>46133</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>46139</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>El poder de la metáfora</t>
+          <t>SCORM</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="E3" s="3" t="n">
-        <v>46133</v>
+        <v>46140</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>46146</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Pensar qué relaciones necesita construir el propio objeto.</t>
-        </is>
-      </c>
+      <c r="G3" s="3" t="n">
+        <v>46147</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Podcast · Frecuencia modulada</t>
+          <t>El poder de la metáfora</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>46147</v>
+        <v>46154</v>
       </c>
       <c r="F4" s="3" t="n">
+        <v>46167</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>46168</v>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>46174</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Tres semanas de cursada y una para el trabajo final.</t>
-        </is>
-      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Podcast · Frecuencia modulada</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>46175</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>46209</v>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Cuatro semanas de cursada y una para el trabajo final.</t>
-        </is>
-      </c>
+        <v>46195</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>46196</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>46202</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n"/>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Laboratorio de simulaciones</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
         <v>4</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>46210</v>
+        <v>46203</v>
       </c>
       <c r="F6" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>46237</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Una semana por movimiento, con sus entregas.</t>
-        </is>
-      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n"/>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SCORM</t>
+          <t>Laboratorio de simulaciones</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>46238</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>46244</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Recorrido breve con demostración y autoevaluación.</t>
-        </is>
-      </c>
+        <v>46265</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G7"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -777,19 +862,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Módulo</t>
@@ -797,17 +885,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Duración (semanas)</t>
+          <t>Cursada (semanas)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Semana inicial</t>
+          <t>Entrega (semanas)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Semana final</t>
+          <t>Total del módulo</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -817,12 +905,27 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Fin de cursada</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Criterio / producción</t>
+          <t>Inicio de entrega</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Fin de entrega</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Foro</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Total de trayectoria</t>
         </is>
       </c>
     </row>
@@ -839,7 +942,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>46126</v>
@@ -847,68 +950,89 @@
       <c r="F2" s="3" t="n">
         <v>46132</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Reconocer los componentes de un objeto de aprendizaje.</t>
-        </is>
-      </c>
+      <c r="G2" s="3" t="n">
+        <v>46133</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>46139</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>El poder de la metáfora</t>
+          <t>SCORM</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="E3" s="3" t="n">
-        <v>46133</v>
+        <v>46140</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>46146</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Pensar qué relaciones necesita construir el propio objeto.</t>
-        </is>
-      </c>
+      <c r="G3" s="3" t="n">
+        <v>46147</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SCORM</t>
+          <t>El poder de la metáfora</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>46147</v>
+        <v>46154</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>46153</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Recorrido breve con demostración y autoevaluación.</t>
-        </is>
-      </c>
+        <v>46167</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>46168</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>46174</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -919,20 +1043,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="65" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Módulo</t>
@@ -940,17 +1066,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Duración (semanas)</t>
+          <t>Cursada (semanas)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Semana inicial</t>
+          <t>Entrega (semanas)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Semana final</t>
+          <t>Total del módulo</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -960,17 +1086,27 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Fin</t>
+          <t>Fin de cursada</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Criterio / producción</t>
+          <t>Inicio de entrega</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Total con base común (semanas)</t>
+          <t>Fin de entrega</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Foro</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Total de trayectoria</t>
         </is>
       </c>
     </row>
@@ -981,27 +1117,33 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E2" s="3" t="n">
-        <v>46154</v>
+        <v>46175</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>46181</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Ficha del episodio, guion didáctico y guion técnico-literario.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>8</v>
+        <v>46195</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>46196</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>46202</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
@@ -1011,27 +1153,33 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>9</v>
-      </c>
       <c r="E3" s="3" t="n">
-        <v>46154</v>
+        <v>46175</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>46188</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Ficha inicial, storyline, sinopsis, escaleta y guion de un episodio.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>9</v>
+        <v>46202</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>46203</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>46209</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
@@ -1044,28 +1192,34 @@
         <v>4</v>
       </c>
       <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E4" s="3" t="n">
-        <v>46154</v>
+        <v>46175</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>46181</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Informe, anteproyecto, prototipo y dossier final a lo largo del módulo.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>8</v>
+        <v>46202</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>46203</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>46209</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Aplicar colores PED también al cronograma Excel
</commit_message>
<xml_diff>
--- a/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
+++ b/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
@@ -24,11 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +39,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,8 +57,13 @@
         <fgColor rgb="005B538E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00132D48"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,11 +71,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00DC5429"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -74,7 +88,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,12 +470,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Criterio</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Definición</t>
         </is>
@@ -467,7 +487,7 @@
           <t>Inicio de ambas trayectorias</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="5" t="n">
         <v>46126</v>
       </c>
     </row>
@@ -595,52 +615,52 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Cursada (semanas)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Entrega (semanas)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Total del módulo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Fin de cursada</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Inicio de entrega</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Fin de entrega</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Foro</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Total de trayectoria</t>
         </is>
@@ -661,16 +681,16 @@
       <c r="D2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="5" t="n">
         <v>46126</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="5" t="n">
         <v>46132</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="5" t="n">
         <v>46133</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="5" t="n">
         <v>46139</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -695,16 +715,16 @@
       <c r="D3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="5" t="n">
         <v>46140</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="5" t="n">
         <v>46146</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="5" t="n">
         <v>46147</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="5" t="n">
         <v>46153</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -729,16 +749,16 @@
       <c r="D4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="5" t="n">
         <v>46154</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="5" t="n">
         <v>46167</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="5" t="n">
         <v>46168</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="5" t="n">
         <v>46174</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -763,16 +783,16 @@
       <c r="D5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="5" t="n">
         <v>46175</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="5" t="n">
         <v>46195</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="5" t="n">
         <v>46196</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="5" t="n">
         <v>46202</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -797,16 +817,16 @@
       <c r="D6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="5" t="n">
         <v>46203</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="5" t="n">
         <v>46230</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="5" t="n">
         <v>46231</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="H6" s="5" t="n">
         <v>46237</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -831,16 +851,16 @@
       <c r="D7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="5" t="n">
         <v>46238</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="5" t="n">
         <v>46265</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G7" s="5" t="n">
         <v>46266</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="5" t="n">
         <v>46272</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -878,52 +898,52 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Cursada (semanas)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Entrega (semanas)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Total del módulo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Fin de cursada</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Inicio de entrega</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Fin de entrega</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Foro</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Total de trayectoria</t>
         </is>
@@ -944,16 +964,16 @@
       <c r="D2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="5" t="n">
         <v>46126</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="5" t="n">
         <v>46132</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="5" t="n">
         <v>46133</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="5" t="n">
         <v>46139</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -978,16 +998,16 @@
       <c r="D3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="5" t="n">
         <v>46140</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="5" t="n">
         <v>46146</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="5" t="n">
         <v>46147</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="5" t="n">
         <v>46153</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1012,16 +1032,16 @@
       <c r="D4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="5" t="n">
         <v>46154</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="5" t="n">
         <v>46167</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="5" t="n">
         <v>46168</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="5" t="n">
         <v>46174</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -1059,52 +1079,52 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Cursada (semanas)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Entrega (semanas)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Total del módulo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Fin de cursada</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Inicio de entrega</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Fin de entrega</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Foro</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Total de trayectoria</t>
         </is>
@@ -1125,16 +1145,16 @@
       <c r="D2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="5" t="n">
         <v>46175</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="5" t="n">
         <v>46195</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="5" t="n">
         <v>46196</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="5" t="n">
         <v>46202</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1161,16 +1181,16 @@
       <c r="D3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="5" t="n">
         <v>46175</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="5" t="n">
         <v>46202</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="5" t="n">
         <v>46203</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="5" t="n">
         <v>46209</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1197,16 +1217,16 @@
       <c r="D4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="5" t="n">
         <v>46175</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="5" t="n">
         <v>46202</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="5" t="n">
         <v>46203</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="5" t="n">
         <v>46209</v>
       </c>
       <c r="I4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Quitar entrega final de SCORM y recalcular trayectorias
</commit_message>
<xml_diff>
--- a/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
+++ b/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
@@ -499,7 +499,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>21 semanas. Anatomía → SCORM → Metáfora → Podcast → Streaming → Simulaciones.</t>
+          <t>20 semanas. Anatomía → SCORM → Metáfora → Podcast → Streaming → Simulaciones.</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>7 semanas: Anatomía, SCORM y Metáfora.</t>
+          <t>6 semanas: Anatomía (2), SCORM (1) y Metáfora (3).</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1 semana adicional en cada módulo, incluida en todos los totales.</t>
+          <t>SCORM no tiene trabajo final. Los otros cinco módulos incluyen una semana adicional de entrega.</t>
         </is>
       </c>
     </row>
@@ -710,10 +710,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>46140</v>
@@ -721,11 +721,9 @@
       <c r="F3" s="5" t="n">
         <v>46146</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>46147</v>
-      </c>
+      <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>46153</v>
+        <v>46146</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -750,16 +748,16 @@
         <v>3</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>46154</v>
+        <v>46147</v>
       </c>
       <c r="F4" s="5" t="n">
+        <v>46160</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>46161</v>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>46167</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>46168</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>46174</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -784,16 +782,16 @@
         <v>4</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>46175</v>
+        <v>46168</v>
       </c>
       <c r="F5" s="5" t="n">
+        <v>46188</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>46195</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>46196</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>46202</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -818,16 +816,16 @@
         <v>5</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>46203</v>
+        <v>46196</v>
       </c>
       <c r="F6" s="5" t="n">
+        <v>46223</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>46224</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>46230</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>46231</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>46237</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -852,16 +850,16 @@
         <v>5</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>46238</v>
+        <v>46231</v>
       </c>
       <c r="F7" s="5" t="n">
+        <v>46258</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>46265</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>46266</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>46272</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -993,10 +991,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>46140</v>
@@ -1004,11 +1002,9 @@
       <c r="F3" s="5" t="n">
         <v>46146</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>46147</v>
-      </c>
+      <c r="G3" s="5" t="n"/>
       <c r="H3" s="5" t="n">
-        <v>46153</v>
+        <v>46146</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -1033,16 +1029,16 @@
         <v>3</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>46154</v>
+        <v>46147</v>
       </c>
       <c r="F4" s="5" t="n">
+        <v>46160</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>46161</v>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>46167</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>46168</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>46174</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -1146,24 +1142,24 @@
         <v>4</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>46175</v>
+        <v>46168</v>
       </c>
       <c r="F2" s="5" t="n">
+        <v>46188</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="H2" s="5" t="n">
         <v>46195</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>46196</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>46202</v>
-      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
@@ -1182,24 +1178,24 @@
         <v>5</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>46175</v>
+        <v>46168</v>
       </c>
       <c r="F3" s="5" t="n">
+        <v>46195</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>46196</v>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>46202</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>46203</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>46209</v>
-      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
@@ -1218,24 +1214,24 @@
         <v>5</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>46175</v>
+        <v>46168</v>
       </c>
       <c r="F4" s="5" t="n">
+        <v>46195</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>46196</v>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>46202</v>
       </c>
-      <c r="G4" s="5" t="n">
-        <v>46203</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>46209</v>
-      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregir totales: el TP ya está incluido en cada módulo
</commit_message>
<xml_diff>
--- a/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
+++ b/version-1-autoasistida/trayectorias/Cronograma_trayectorias_OA.xlsx
@@ -14,9 +14,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Criterios'!$A$1:$B$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Certificación completa'!$A$1:$J$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Base común modular'!$A$1:$J$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opciones modulares'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Certificación completa'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Base común modular'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Opciones modulares'!$A$1:$H$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,10 +24,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,23 +40,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="005B538E"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -80,21 +71,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,12 +455,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Criterio</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Definición</t>
         </is>
@@ -484,82 +469,82 @@
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inicio de ambas trayectorias</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="n">
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>46126</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Certificación completa</t>
+          <t>Duración</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>20 semanas. Anatomía → SCORM → Metáfora → Podcast → Streaming → Simulaciones.</t>
+          <t>El TP está incluido en el total de cada módulo. No se suman semanas.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Base común modular</t>
+          <t>Certificación completa</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>6 semanas: Anatomía (2), SCORM (1) y Metáfora (3).</t>
+          <t>15 semanas. Diseñar un objeto de aprendizaje propio.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Entrega final</t>
+          <t>Base común</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SCORM no tiene trabajo final. Los otros cinco módulos incluyen una semana adicional de entrega.</t>
+          <t>Anatomía (1) → SCORM (1) → Metáfora (2): 4 semanas.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Foros</t>
+          <t>SCORM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Todos los módulos incluyen un foro de intercambio.</t>
+          <t>Segundo lugar, con foro y sin trabajo final.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de certificación</t>
+          <t>Foros</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Diseño de un objeto de aprendizaje propio.</t>
+          <t>Todos los módulos tienen foro de intercambio.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Articulación del proyecto</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Pendiente de definir su relación con trabajos de módulo; sin semana integradora adicional.</t>
+          <t>Última semana dentro del módulo. Anatomía integra cursada y TP en la misma semana.</t>
         </is>
       </c>
     </row>
@@ -571,7 +556,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>No contemplados; semanas consecutivas de martes a lunes.</t>
+          <t>No contemplados.</t>
         </is>
       </c>
     </row>
@@ -599,70 +584,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Cursada (semanas)</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Entrega (semanas)</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Total del módulo</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total semanas (TP incluido)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Fin de cursada</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Inicio de entrega</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Fin de entrega</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Inicio TP (incluido)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fin TP (incluido)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foro</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Total de trayectoria</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Total trayectoria</t>
         </is>
       </c>
     </row>
@@ -675,30 +648,24 @@
       <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" s="5" t="n">
+      <c r="C2" s="3" t="n">
         <v>46126</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="D2" s="3" t="n">
         <v>46132</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>46133</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>46139</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="n">
+        <v>46126</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>46132</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -709,28 +676,20 @@
       <c r="B3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>46146</v>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n">
-        <v>46146</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="n">
+        <v>46133</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -741,30 +700,24 @@
       <c r="B4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="5" t="n">
+      <c r="C4" s="3" t="n">
+        <v>46140</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>46147</v>
       </c>
-      <c r="F4" s="5" t="n">
-        <v>46160</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>46161</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>46167</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -775,30 +728,24 @@
       <c r="B5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E5" s="5" t="n">
+      <c r="C5" s="3" t="n">
+        <v>46154</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>46168</v>
       </c>
-      <c r="F5" s="5" t="n">
-        <v>46188</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>46195</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="n">
+        <v>46174</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -809,30 +756,24 @@
       <c r="B6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" s="5" t="n">
+      <c r="C6" s="3" t="n">
+        <v>46175</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>46196</v>
       </c>
-      <c r="F6" s="5" t="n">
-        <v>46223</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>46224</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>46230</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="n">
+        <v>46202</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -843,33 +784,27 @@
       <c r="B7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>46231</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>46258</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>46265</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="n">
+        <v>46203</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>46224</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:H7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -880,70 +815,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Cursada (semanas)</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Entrega (semanas)</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Total del módulo</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total semanas (TP incluido)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Fin de cursada</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Inicio de entrega</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Fin de entrega</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Inicio TP (incluido)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fin TP (incluido)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foro</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Total de trayectoria</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Total trayectoria</t>
         </is>
       </c>
     </row>
@@ -956,30 +879,24 @@
       <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" s="5" t="n">
+      <c r="C2" s="3" t="n">
         <v>46126</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="D2" s="3" t="n">
         <v>46132</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>46133</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>46139</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="n">
+        <v>46126</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>46132</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -990,28 +907,20 @@
       <c r="B3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>46146</v>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n">
-        <v>46146</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="n">
+        <v>46133</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1022,33 +931,27 @@
       <c r="B4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="5" t="n">
+      <c r="C4" s="3" t="n">
+        <v>46140</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>46147</v>
       </c>
-      <c r="F4" s="5" t="n">
-        <v>46160</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>46161</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>46167</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="n">
+        <v>46153</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:H4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1059,70 +962,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Cursada (semanas)</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Entrega (semanas)</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Total del módulo</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total semanas (TP incluido)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Inicio</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Fin de cursada</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Inicio de entrega</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Fin de entrega</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Inicio TP (incluido)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fin TP (incluido)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foro</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Total de trayectoria</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Total trayectoria</t>
         </is>
       </c>
     </row>
@@ -1135,31 +1026,25 @@
       <c r="B2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E2" s="5" t="n">
+      <c r="C2" s="3" t="n">
+        <v>46154</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>46168</v>
       </c>
-      <c r="F2" s="5" t="n">
-        <v>46188</v>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>46189</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>46195</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="n">
+        <v>46174</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>10</v>
+      <c r="H2" s="2" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="3" ht="44" customHeight="1">
@@ -1171,31 +1056,25 @@
       <c r="B3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>46168</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>46195</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>46196</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>46202</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="n">
+        <v>46154</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>46181</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>46175</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>46181</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
-        <v>11</v>
+      <c r="H3" s="2" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="4" ht="44" customHeight="1">
@@ -1207,35 +1086,29 @@
       <c r="B4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>46168</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>46195</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>46196</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>46202</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="n">
+        <v>46154</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>46181</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>46175</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>46181</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
-        <v>11</v>
+      <c r="H4" s="2" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J4"/>
+  <autoFilter ref="A1:H4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>